<commit_message>
Sales & Returns updated
</commit_message>
<xml_diff>
--- a/input/Chiraath - Business Summary.xlsx
+++ b/input/Chiraath - Business Summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E4BE83-2814-4547-B274-C644FA88F445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FA1AA75-205A-564E-82FA-2065E58215DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3555" uniqueCount="1402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3559" uniqueCount="1402">
   <si>
     <t>Notes:</t>
   </si>
@@ -4139,9 +4139,6 @@
     <t>Beige and Dark Green, Beige and Maroon, Mustard Yellow and Dark Green, Magenta Pink and Royal Blue</t>
   </si>
   <si>
-    <t>Teal Blue and Silver, Royal Blue and Silver, Teal Green and Magenta Pink</t>
-  </si>
-  <si>
     <t>Prabha Chidambaram - Green, Wine red returned, Blue - Lakshmi</t>
   </si>
   <si>
@@ -4269,6 +4266,9 @@
   </si>
   <si>
     <t>Chocolate Brown.</t>
+  </si>
+  <si>
+    <t>Teal Blue and Silver, Royal Blue and Silver</t>
   </si>
 </sst>
 </file>
@@ -5285,7 +5285,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>80</c:v>
+                  <c:v>78</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>62</c:v>
@@ -5618,7 +5618,7 @@
                   <c:v>67003</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-194924.99333333335</c:v>
+                  <c:v>-196630.99333333335</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -5957,7 +5957,7 @@
                   <c:v>45848</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-8192</c:v>
+                  <c:v>-9898</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -6557,7 +6557,7 @@
                   <c:v>33250</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>17152</c:v>
+                  <c:v>18858</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -7018,7 +7018,7 @@
                   <c:v>476</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>145</c:v>
+                  <c:v>143</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8210,7 +8210,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>594003</v>
+        <v>592297</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>568431</v>
+        <v>570831</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -8259,7 +8259,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-25572</v>
+        <v>-21466</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>44413.66</v>
+        <v>44982.32666666666</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -8304,7 +8304,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>61044.67</v>
+        <v>59907.336666666655</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -8314,7 +8314,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-105458.33</v>
+        <v>-104889.66333333334</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -8357,11 +8357,11 @@
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>198001</v>
+        <v>197432.33333333334</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>62717</v>
+        <v>63285.666666666657</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8369,11 +8369,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>44413.66</v>
+        <v>44982.32666666666</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹44,414</v>
+        <v>Receive ₹44,982</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -8383,15 +8383,15 @@
       </c>
       <c r="B19" s="12">
         <f>PartnerShares!B9</f>
-        <v>300685</v>
+        <v>298979</v>
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>198001</v>
+        <v>197432.33333333334</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>102684</v>
+        <v>101546.66666666666</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8399,11 +8399,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>61044.67</v>
+        <v>59907.336666666655</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹61,045</v>
+        <v>Receive ₹59,907</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -8417,11 +8417,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>198001</v>
+        <v>197432.33333333334</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-165401</v>
+        <v>-164832.33333333334</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8429,11 +8429,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-105458.33</v>
+        <v>-104889.66333333334</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹105,458</v>
+        <v>Pay ₹104,890</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -8471,15 +8471,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>495678</v>
+        <v>498078</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>189514.89539999998</v>
+        <v>190315.05539999998</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>306163.10460000002</v>
+        <v>307762.94460000005</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -8487,11 +8487,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>168853.07860000001</v>
+        <v>170452.91860000003</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹168,853</v>
+        <v>Pay ₹170,453</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -8505,11 +8505,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>189401.20920000001</v>
+        <v>190200.88920000001</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-130178.20920000001</v>
+        <v>-130977.88920000001</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -8517,11 +8517,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-58591.167200000011</v>
+        <v>-59390.847200000004</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹58,591</v>
+        <v>Receive ₹59,391</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -8535,11 +8535,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>189514.89539999998</v>
+        <v>190315.05539999998</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-176984.89539999998</v>
+        <v>-177785.05539999998</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -8547,11 +8547,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-111261.91139999997</v>
+        <v>-112062.07139999997</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹111,262</v>
+        <v>Receive ₹112,062</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46278</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -8672,14 +8672,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>594003</v>
+        <v>592297</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>568431</v>
+        <v>570831</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -8688,14 +8688,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-25572</v>
+        <v>-21466</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>-139293.79333333333</v>
+        <v>-140999.79333333333</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8882,7 +8882,7 @@
       </c>
       <c r="B18" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A18)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>-8192</v>
+        <v>-9898</v>
       </c>
       <c r="C18" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$993,"MMM")=$A18)*(YEAR(Sales!$A$2:$A$993)=$B$7)*Sales!$C$2:$C$993),0)</f>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="D18" s="21">
         <f t="shared" si="0"/>
-        <v>17152</v>
+        <v>18858</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15" customHeight="1">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8998,7 +8998,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$475=J48)*(INVENTORY!$D$2:$D$475)*(INVENTORY!$G$2:$G$475))</f>
-        <v>-194924.99333333335</v>
+        <v>-196630.99333333335</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -10707,7 +10707,7 @@
         <v>-4202</v>
       </c>
       <c r="D115" s="39" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="15" customHeight="1">
@@ -10721,7 +10721,7 @@
         <v>-1620</v>
       </c>
       <c r="D116" s="36" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="15" customHeight="1">
@@ -10735,7 +10735,7 @@
         <v>-603</v>
       </c>
       <c r="D117" s="39" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="15" customHeight="1">
@@ -10749,14 +10749,22 @@
         <v>-1911</v>
       </c>
       <c r="D118" s="36" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="15" customHeight="1">
-      <c r="A119" s="38"/>
-      <c r="B119" s="39"/>
-      <c r="C119" s="40"/>
-      <c r="D119" s="39"/>
+      <c r="A119" s="38">
+        <v>46277</v>
+      </c>
+      <c r="B119" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="C119" s="40">
+        <v>-1706</v>
+      </c>
+      <c r="D119" s="39" t="s">
+        <v>1382</v>
+      </c>
     </row>
     <row r="120" spans="1:4" ht="15" customHeight="1">
       <c r="A120" s="35"/>
@@ -19293,7 +19301,7 @@
       <c r="F265" s="46"/>
       <c r="G265" s="46"/>
       <c r="H265" s="46" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="I265" s="45" t="s">
         <v>148</v>
@@ -19364,7 +19372,7 @@
       <c r="F268" s="44"/>
       <c r="G268" s="44"/>
       <c r="H268" s="44" t="s">
-        <v>1397</v>
+        <v>1396</v>
       </c>
       <c r="I268" s="44" t="s">
         <v>356</v>
@@ -19950,7 +19958,7 @@
         <v>46229</v>
       </c>
       <c r="B292" s="45" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="C292" s="85">
         <v>3600</v>
@@ -19960,7 +19968,7 @@
       <c r="F292" s="46"/>
       <c r="G292" s="46"/>
       <c r="H292" s="46" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="I292" s="45" t="s">
         <v>356</v>
@@ -20227,7 +20235,7 @@
       <c r="F303" s="44"/>
       <c r="G303" s="44"/>
       <c r="H303" s="44" t="s">
-        <v>1367</v>
+        <v>1366</v>
       </c>
       <c r="I303" s="44" t="s">
         <v>148</v>
@@ -20252,7 +20260,7 @@
       <c r="F304" s="46"/>
       <c r="G304" s="46"/>
       <c r="H304" s="46" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
       <c r="I304" s="45" t="s">
         <v>148</v>
@@ -20838,7 +20846,7 @@
         <v>46275</v>
       </c>
       <c r="B328" s="44" t="s">
-        <v>1368</v>
+        <v>1367</v>
       </c>
       <c r="C328" s="83">
         <v>1380</v>
@@ -20852,7 +20860,7 @@
       <c r="F328" s="44"/>
       <c r="G328" s="44"/>
       <c r="H328" s="44" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="I328" s="44" t="s">
         <v>148</v>
@@ -20868,15 +20876,19 @@
       <c r="C329" s="85">
         <v>2400</v>
       </c>
-      <c r="D329" s="45"/>
-      <c r="E329" s="45"/>
+      <c r="D329" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="E329" s="45" t="s">
+        <v>49</v>
+      </c>
       <c r="F329" s="46"/>
       <c r="G329" s="46"/>
       <c r="H329" s="46" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
       <c r="I329" s="45" t="s">
-        <v>356</v>
+        <v>148</v>
       </c>
     </row>
     <row r="330" spans="1:9" ht="14">
@@ -20884,7 +20896,7 @@
         <v>46275</v>
       </c>
       <c r="B330" s="44" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
       <c r="C330" s="83">
         <v>1450</v>
@@ -20898,7 +20910,7 @@
       <c r="F330" s="44"/>
       <c r="G330" s="44"/>
       <c r="H330" s="44" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="I330" s="44" t="s">
         <v>148</v>
@@ -20909,7 +20921,7 @@
         <v>46275</v>
       </c>
       <c r="B331" s="45" t="s">
-        <v>1379</v>
+        <v>1378</v>
       </c>
       <c r="C331" s="85">
         <v>950</v>
@@ -20923,7 +20935,7 @@
       <c r="F331" s="46"/>
       <c r="G331" s="46"/>
       <c r="H331" s="46" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="I331" s="45" t="s">
         <v>148</v>
@@ -20948,7 +20960,7 @@
       <c r="F332" s="44"/>
       <c r="G332" s="44"/>
       <c r="H332" s="44" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="I332" s="44" t="s">
         <v>148</v>
@@ -20973,7 +20985,7 @@
       <c r="F333" s="46"/>
       <c r="G333" s="46"/>
       <c r="H333" s="46" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
       <c r="I333" s="45" t="s">
         <v>148</v>
@@ -20990,7 +21002,7 @@
         <v>1380</v>
       </c>
       <c r="D334" s="44" t="s">
-        <v>1390</v>
+        <v>1389</v>
       </c>
       <c r="E334" s="44" t="s">
         <v>49</v>
@@ -20998,7 +21010,7 @@
       <c r="F334" s="44"/>
       <c r="G334" s="44"/>
       <c r="H334" s="44" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="I334" s="44" t="s">
         <v>148</v>
@@ -28847,7 +28859,7 @@
         <v>0</v>
       </c>
       <c r="L78" s="52" t="s">
-        <v>1376</v>
+        <v>1375</v>
       </c>
       <c r="M78" s="52"/>
       <c r="N78" s="52" t="s">
@@ -29167,14 +29179,14 @@
         <v>450</v>
       </c>
       <c r="L84" s="52" t="s">
-        <v>1374</v>
+        <v>1373</v>
       </c>
       <c r="M84" s="52"/>
       <c r="N84" s="52" t="s">
         <v>589</v>
       </c>
       <c r="O84" s="52" t="s">
-        <v>1373</v>
+        <v>1372</v>
       </c>
       <c r="P84" s="52"/>
       <c r="Q84" s="52"/>
@@ -29273,14 +29285,14 @@
         <v>1045</v>
       </c>
       <c r="L86" s="52" t="s">
-        <v>1377</v>
+        <v>1376</v>
       </c>
       <c r="M86" s="52"/>
       <c r="N86" s="52" t="s">
         <v>589</v>
       </c>
       <c r="O86" s="52" t="s">
-        <v>1378</v>
+        <v>1377</v>
       </c>
       <c r="P86" s="52"/>
       <c r="Q86" s="52"/>
@@ -35646,7 +35658,7 @@
         <v>589</v>
       </c>
       <c r="P194" s="47" t="s">
-        <v>1381</v>
+        <v>1380</v>
       </c>
       <c r="S194" s="47"/>
       <c r="T194" s="47"/>
@@ -35839,14 +35851,14 @@
         <v>934</v>
       </c>
       <c r="L198" s="55" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
       <c r="M198" s="55"/>
       <c r="N198" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P198" s="47" t="s">
-        <v>1385</v>
+        <v>1384</v>
       </c>
       <c r="S198" s="47"/>
       <c r="T198" s="47"/>
@@ -35958,7 +35970,7 @@
         <v>996</v>
       </c>
       <c r="B201" s="55" t="s">
-        <v>1366</v>
+        <v>1365</v>
       </c>
       <c r="C201" s="55" t="s">
         <v>95</v>
@@ -35999,7 +36011,7 @@
         <v>589</v>
       </c>
       <c r="P201" s="47" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="S201" s="47"/>
       <c r="T201" s="47"/>
@@ -36145,7 +36157,7 @@
         <v>0</v>
       </c>
       <c r="L204" s="55" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="M204" s="55"/>
       <c r="N204" s="47" t="s">
@@ -36545,7 +36557,7 @@
         <v>2775</v>
       </c>
       <c r="L212" s="55" t="s">
-        <v>1382</v>
+        <v>1381</v>
       </c>
       <c r="M212" s="55"/>
       <c r="N212" s="47" t="s">
@@ -36577,11 +36589,11 @@
         <v>1</v>
       </c>
       <c r="G213" s="66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H213" s="65">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I213" s="65">
         <f>IF(D213&lt;&gt;"",D213,IFERROR(E213/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -36593,7 +36605,7 @@
       </c>
       <c r="K213" s="65">
         <f t="shared" si="14"/>
-        <v>3340</v>
+        <v>2505</v>
       </c>
       <c r="L213" s="52" t="s">
         <v>1301</v>
@@ -36849,7 +36861,7 @@
         <v>761</v>
       </c>
       <c r="L218" s="55" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="M218" s="55"/>
       <c r="N218" s="47" t="s">
@@ -37351,7 +37363,7 @@
         <v>0</v>
       </c>
       <c r="L228" s="52" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="M228" s="52"/>
       <c r="N228" s="47" t="s">
@@ -37704,7 +37716,7 @@
         <v>734</v>
       </c>
       <c r="L235" s="55" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="M235" s="55"/>
       <c r="N235" s="47" t="s">
@@ -37860,7 +37872,7 @@
         <v>677</v>
       </c>
       <c r="P238" s="86" t="s">
-        <v>1384</v>
+        <v>1383</v>
       </c>
       <c r="S238" s="47"/>
       <c r="T238" s="47"/>
@@ -38863,7 +38875,7 @@
         <v>1304</v>
       </c>
       <c r="B250" s="52" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="C250" s="52" t="s">
         <v>96</v>
@@ -38905,7 +38917,7 @@
         <v>1307</v>
       </c>
       <c r="P250" s="86" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="S250" s="47"/>
       <c r="T250" s="47"/>
@@ -38915,7 +38927,7 @@
         <v>1308</v>
       </c>
       <c r="B251" s="55" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
       <c r="C251" s="55" t="s">
         <v>96</v>
@@ -38957,7 +38969,7 @@
         <v>1309</v>
       </c>
       <c r="P251" s="86" t="s">
-        <v>1396</v>
+        <v>1395</v>
       </c>
       <c r="S251" s="47"/>
       <c r="T251" s="47"/>
@@ -38967,7 +38979,7 @@
         <v>1310</v>
       </c>
       <c r="B252" s="52" t="s">
-        <v>1394</v>
+        <v>1393</v>
       </c>
       <c r="C252" s="52" t="s">
         <v>96</v>
@@ -39009,7 +39021,7 @@
         <v>1309</v>
       </c>
       <c r="P252" s="86" t="s">
-        <v>1398</v>
+        <v>1397</v>
       </c>
       <c r="S252" s="47"/>
       <c r="T252" s="47"/>
@@ -39019,7 +39031,7 @@
         <v>1311</v>
       </c>
       <c r="B253" s="55" t="s">
-        <v>1395</v>
+        <v>1394</v>
       </c>
       <c r="C253" s="55" t="s">
         <v>96</v>
@@ -39061,7 +39073,7 @@
         <v>1307</v>
       </c>
       <c r="P253" s="86" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="S253" s="47"/>
       <c r="T253" s="47"/>
@@ -39154,7 +39166,7 @@
         <v>0</v>
       </c>
       <c r="L255" s="55" t="s">
-        <v>1391</v>
+        <v>1390</v>
       </c>
       <c r="M255" s="55"/>
       <c r="N255" s="47" t="s">
@@ -39374,11 +39386,11 @@
         <v>0</v>
       </c>
       <c r="G260" s="66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H260" s="65">
         <f t="shared" si="18"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I260" s="65">
         <f>IF(D260&lt;&gt;"",D260,IFERROR(E260/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -39390,7 +39402,7 @@
       </c>
       <c r="K260" s="65">
         <f t="shared" si="20"/>
-        <v>2613</v>
+        <v>1742</v>
       </c>
       <c r="L260" s="52"/>
       <c r="M260" s="52"/>
@@ -39398,7 +39410,7 @@
         <v>677</v>
       </c>
       <c r="P260" s="86" t="s">
-        <v>1358</v>
+        <v>1401</v>
       </c>
       <c r="S260" s="47"/>
       <c r="T260" s="47"/>
@@ -39496,7 +39508,7 @@
         <v>677</v>
       </c>
       <c r="P262" s="86" t="s">
-        <v>1392</v>
+        <v>1391</v>
       </c>
       <c r="S262" s="47"/>
       <c r="T262" s="47"/>
@@ -45713,11 +45725,11 @@
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>198001</v>
+        <v>197432.33333333334</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>62717</v>
+        <v>63285.666666666657</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -45725,7 +45737,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>62717</v>
+        <v>63285.666666666657</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -45733,7 +45745,7 @@
       </c>
       <c r="H8" s="73">
         <f>F8-G8</f>
-        <v>44413.66</v>
+        <v>44982.32666666666</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -45742,15 +45754,15 @@
       </c>
       <c r="B9" s="11">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A9,Purchases!$C:$C),0)</f>
-        <v>300685</v>
+        <v>298979</v>
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>198001</v>
+        <v>197432.33333333334</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>102684</v>
+        <v>101546.66666666666</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -45758,7 +45770,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>102684</v>
+        <v>101546.66666666666</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -45766,7 +45778,7 @@
       </c>
       <c r="H9" s="74">
         <f>F9-G9</f>
-        <v>61044.67</v>
+        <v>59907.336666666655</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -45779,11 +45791,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>198001</v>
+        <v>197432.33333333334</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-165401</v>
+        <v>-164832.33333333334</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -45791,7 +45803,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-165401</v>
+        <v>-164832.33333333334</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -45799,7 +45811,7 @@
       </c>
       <c r="H10" s="73">
         <f>F10-G10</f>
-        <v>-105458.33</v>
+        <v>-104889.66333333334</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="75" customFormat="1" ht="15.75" customHeight="1">
@@ -46216,7 +46228,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>495678</v>
+        <v>498078</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -46224,11 +46236,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>189514.89539999998</v>
+        <v>190315.05539999998</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>306163.10460000002</v>
+        <v>307762.94460000005</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -46236,7 +46248,7 @@
       </c>
       <c r="G4" s="73">
         <f>E4+F4</f>
-        <v>168853.07860000001</v>
+        <v>170452.91860000003</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -46253,11 +46265,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>189401.20920000001</v>
+        <v>190200.88920000001</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-130178.20920000001</v>
+        <v>-130977.88920000001</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -46265,7 +46277,7 @@
       </c>
       <c r="G5" s="74">
         <f>E5+F5</f>
-        <v>-58591.167200000011</v>
+        <v>-59390.847200000004</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -46282,11 +46294,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>189514.89539999998</v>
+        <v>190315.05539999998</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-176984.89539999998</v>
+        <v>-177785.05539999998</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -46294,7 +46306,7 @@
       </c>
       <c r="G6" s="73">
         <f>E6+F6</f>
-        <v>-111261.91139999997</v>
+        <v>-112062.07139999997</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>